<commit_message>
refactor: update pricing, sizing calculations, and documentation for AWS Bedrock and infrastructure components
</commit_message>
<xml_diff>
--- a/G03_baogia.xlsx
+++ b/G03_baogia.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaoGia" sheetId="1" r:id="Rdb444af4e6b144fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BangChung" sheetId="2" r:id="Rfe403e08cc7547eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaoGia" sheetId="1" r:id="R5c2ee85111714dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BangChung" sheetId="2" r:id="Rfa92fa14de614999"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -359,16 +359,16 @@
         <x:v>llm</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
-        <x:v>LLM serving và sinh ảnh theo usage</x:v>
+        <x:v>LLM serving theo APAC Geo Cross-Region</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
-        <x:v>Bedrock Nova Lite Cấp 1-3: 5,324.0M input × 0.081 + 765.6M output × 0.324; Nova Pro Cấp 4-5: 1,364.0M × 1.08 + 220.0M × 4.32; 90,000 ảnh × 0.01 USD/ảnh; Singapore.</x:v>
+        <x:v>Bedrock apac.amazon.nova-lite-v1:0: 6,512M input × 0.063 + 950.4M output × 0.252; apac.amazon.nova-pro-v1:0: 4,576M × 0.84 + 739.2M × 3.36 USD/1M; agent steps C3=2, C4=3, C5=4; ảnh render SVG/HTML.</x:v>
       </x:c>
       <x:c r="D3" s="8" t="n">
-        <x:v>4002.82</x:v>
+        <x:v>6977.31</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
-        <x:v>E01</x:v>
+        <x:v>E01; E18; E19; E20</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -379,13 +379,13 @@
         <x:v>Embedding và vector hoá tài liệu</x:v>
       </x:c>
       <x:c r="C4" s="7" t="str">
-        <x:v>Bedrock embedding batch cho 50M token/tháng × 0.0001 USD/1K token; index pgvector dùng chung Aurora; ap-southeast-1.</x:v>
+        <x:v>Titan Text Embeddings V2: 50M corpus token + 1,760M query token = 1,810M × 0.02 USD/1M; vector index pgvector trong Aurora; Singapore endpoint.</x:v>
       </x:c>
       <x:c r="D4" s="8" t="n">
-        <x:v>5</x:v>
+        <x:v>36.2</x:v>
       </x:c>
       <x:c r="E4" s="7" t="str">
-        <x:v>E01; E06</x:v>
+        <x:v>E06; E23</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -393,16 +393,16 @@
         <x:v>gateway</x:v>
       </x:c>
       <x:c r="B5" s="7" t="str">
-        <x:v>HTTP API và LLM gateway</x:v>
+        <x:v>HTTP API, quota và budget gateway</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>API Gateway HTTP API 1.76M request × 1.00 USD/M; routing, retry, quota và token log chạy trong app Fargate; ap-southeast-1.</x:v>
+        <x:v>API Gateway HTTP API 1.76M × 1.00 USD/M + 10 budget alarms × 0.10 USD; routing, retry, quota và token log chạy trong app; ap-southeast-1.</x:v>
       </x:c>
       <x:c r="D5" s="8" t="n">
-        <x:v>1.76</x:v>
+        <x:v>2.76</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
-        <x:v>E03</x:v>
+        <x:v>E03; E13</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -498,10 +498,10 @@
         <x:v>Workspace riêng và file</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>S3 Standard 6,000GB × 0.023 USD/GB-month; prefix per user, SSE-KMS, lifecycle cho bản cũ; staging 100GB nằm trong cùng bucket.</x:v>
+        <x:v>S3 Standard production 6,000GB + staging 100GB = 6,100GB × 0.023 USD/GB-month; prefix per user, SSE-KMS, lifecycle cho bản cũ.</x:v>
       </x:c>
       <x:c r="D11" s="8" t="n">
-        <x:v>138</x:v>
+        <x:v>140.3</x:v>
       </x:c>
       <x:c r="E11" s="7" t="str">
         <x:v>E07</x:v>
@@ -631,16 +631,16 @@
         <x:v>network</x:v>
       </x:c>
       <x:c r="B19" s="7" t="str">
-        <x:v>VPC, NAT, egress, WAF, private path</x:v>
+        <x:v>VPC, NAT, WAF và Bedrock PrivateLink</x:v>
       </x:c>
       <x:c r="C19" s="7" t="str">
-        <x:v>2 NAT gateway × 730h × 0.059 USD/h + 50GB processing × 0.059 USD/GB + WAF 1 ACL + 2 rule + 1.76M request; private subnets, no sandbox egress.</x:v>
+        <x:v>2 NAT × 730h × 0.059 + 50GB NAT × 0.059 + WAF 1 ACL/2 rule/1.76M request + 1 Bedrock interface endpoint/AZ × 2 AZ × 730h × 0.01 + 50GB endpoint × 0.01; private subnets, sandbox no egress.</x:v>
       </x:c>
       <x:c r="D19" s="8" t="n">
-        <x:v>103.1</x:v>
+        <x:v>118.2</x:v>
       </x:c>
       <x:c r="E19" s="7" t="str">
-        <x:v>E11; E12</x:v>
+        <x:v>E11; E12; E17</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -705,7 +705,7 @@
         <x:v>10% × subtotal trước dự phòng; bao phủ biến động request, log và egress; tính từ các dòng chi phí bên trên.</x:v>
       </x:c>
       <x:c r="D23" s="8" t="n">
-        <x:v>1061.34</x:v>
+        <x:v>1363.75</x:v>
       </x:c>
       <x:c r="E23" s="7" t="str">
         <x:v>NA</x:v>
@@ -723,7 +723,7 @@
       </x:c>
       <x:c r="D24" s="12" t="n">
         <x:f>SUM(D2:D23)</x:f>
-        <x:v>11674.740000000002</x:v>
+        <x:v>15001.24</x:v>
       </x:c>
       <x:c r="E24" s="11" t="str"/>
     </x:row>
@@ -1032,6 +1032,125 @@
         <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="7" t="str">
+        <x:v>E17</x:v>
+      </x:c>
+      <x:c r="B18" s="7" t="str">
+        <x:v>AWS PrivateLink interface endpoint pricing</x:v>
+      </x:c>
+      <x:c r="C18" s="7" t="str">
+        <x:v>https://aws.amazon.com/privatelink/pricing/</x:v>
+      </x:c>
+      <x:c r="D18" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="7" t="str">
+        <x:v>E18</x:v>
+      </x:c>
+      <x:c r="B19" s="7" t="str">
+        <x:v>Nova Lite APAC Geo inference profile and supported destinations</x:v>
+      </x:c>
+      <x:c r="C19" s="7" t="str">
+        <x:v>https://docs.aws.amazon.com/bedrock/latest/userguide/model-card-amazon-nova-lite.html</x:v>
+      </x:c>
+      <x:c r="D19" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E19" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="7" t="str">
+        <x:v>E19</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="str">
+        <x:v>Nova Pro APAC Geo inference profile and supported destinations</x:v>
+      </x:c>
+      <x:c r="C20" s="7" t="str">
+        <x:v>https://docs.aws.amazon.com/bedrock/latest/userguide/model-card-amazon-nova-pro.html</x:v>
+      </x:c>
+      <x:c r="D20" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E20" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="7" t="str">
+        <x:v>E20</x:v>
+      </x:c>
+      <x:c r="B21" s="7" t="str">
+        <x:v>Titan Image Generator G1 v2 lifecycle, region and endpoint support</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="str">
+        <x:v>https://docs.aws.amazon.com/bedrock/latest/userguide/model-card-amazon-titan-image-generator-g1-v2.html</x:v>
+      </x:c>
+      <x:c r="D21" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E21" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="7" t="str">
+        <x:v>E21</x:v>
+      </x:c>
+      <x:c r="B22" s="7" t="str">
+        <x:v>Claude Opus 5.5 benchmark reference and public token price</x:v>
+      </x:c>
+      <x:c r="C22" s="7" t="str">
+        <x:v>https://www.anthropic.com/claude-opus-5-5</x:v>
+      </x:c>
+      <x:c r="D22" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E22" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="7" t="str">
+        <x:v>E22</x:v>
+      </x:c>
+      <x:c r="B23" s="7" t="str">
+        <x:v>Claude Sonnet 5.5 benchmark fallback reference and public token price</x:v>
+      </x:c>
+      <x:c r="C23" s="7" t="str">
+        <x:v>https://www.anthropic.com/claude-sonnet-5-5</x:v>
+      </x:c>
+      <x:c r="D23" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E23" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="7" t="str">
+        <x:v>E23</x:v>
+      </x:c>
+      <x:c r="B24" s="7" t="str">
+        <x:v>Titan Text Embeddings V2 price and model availability</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="str">
+        <x:v>https://aws.amazon.com/blogs/machine-learning/get-started-with-amazon-titan-text-embeddings-v2-a-new-state-of-the-art-embedding-model-on-aws/</x:v>
+      </x:c>
+      <x:c r="D24" s="7" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="str">
+        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
refactor: separate model calls from requests
</commit_message>
<xml_diff>
--- a/G03_baogia.xlsx
+++ b/G03_baogia.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaoGia" sheetId="1" r:id="R5c2ee85111714dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BangChung" sheetId="2" r:id="Rfa92fa14de614999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaoGia" sheetId="1" r:id="Re043ed89c69049e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BangChung" sheetId="2" r:id="Rc66ec0a9f45f4edb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,13 +362,13 @@
         <x:v>LLM serving theo APAC Geo Cross-Region</x:v>
       </x:c>
       <x:c r="C3" s="7" t="str">
-        <x:v>Bedrock apac.amazon.nova-lite-v1:0: 6,512M input × 0.063 + 950.4M output × 0.252; apac.amazon.nova-pro-v1:0: 4,576M × 0.84 + 739.2M × 3.36 USD/1M; agent steps C3=2, C4=3, C5=4; ảnh render SVG/HTML.</x:v>
+        <x:v>Giả định cần đo: Lite C1–3 = 6,512M input × 0.063 + 950.4M output × 0.252; Pro C4–5 = 3,124M input × 0.84 + 501.6M output × 3.36 USD/1M; tổng 2.376M model calls; image tách riêng. PENDING_VERIFICATION giá APAC.</x:v>
       </x:c>
       <x:c r="D3" s="8" t="n">
-        <x:v>6977.31</x:v>
+        <x:v>4959.2928</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
-        <x:v>E01; E18; E19; E20</x:v>
+        <x:v>E01; E18; E19; PENDING_VERIFICATION</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -532,13 +532,13 @@
         <x:v>Sandbox chạy code agent</x:v>
       </x:c>
       <x:c r="C13" s="7" t="str">
-        <x:v>Fargate ARM sandbox 400,000 lượt × 30s × (0.25 vCPU × 0.0000089944 + 0.5GB × 0.0000009889) USD/s; 60 task slots, no egress, TTL 30s.</x:v>
+        <x:v>Fargate ARM ap-southeast-1; 400,000 lượt × billing minimum 60s × (0.25 vCPU × 0.0000089944 + 0.5GB × 0.0000009889) USD/s; workload TTL 30s, no egress. PENDING_VERIFICATION SKU.</x:v>
       </x:c>
       <x:c r="D13" s="8" t="n">
-        <x:v>35.98</x:v>
+        <x:v>65.8332</x:v>
       </x:c>
       <x:c r="E13" s="7" t="str">
-        <x:v>E02; E11</x:v>
+        <x:v>E02; E11; PENDING_VERIFICATION</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -705,7 +705,7 @@
         <x:v>10% × subtotal trước dự phòng; bao phủ biến động request, log và egress; tính từ các dòng chi phí bên trên.</x:v>
       </x:c>
       <x:c r="D23" s="8" t="n">
-        <x:v>1363.75</x:v>
+        <x:v>1164.93</x:v>
       </x:c>
       <x:c r="E23" s="7" t="str">
         <x:v>NA</x:v>
@@ -719,13 +719,15 @@
         <x:v>Tổng hạ tầng + vận hành</x:v>
       </x:c>
       <x:c r="C24" s="11" t="str">
-        <x:v>Tổng các dòng chi phí; USD/tháng, chưa VAT; 2,000 DAU.</x:v>
+        <x:v>Tổng các dòng chi phí; USD/tháng, chưa VAT; 2,000 DAU; working estimate có PENDING_VERIFICATION.</x:v>
       </x:c>
       <x:c r="D24" s="12" t="n">
         <x:f>SUM(D2:D23)</x:f>
-        <x:v>15001.24</x:v>
-      </x:c>
-      <x:c r="E24" s="11" t="str"/>
+        <x:v>12814.256000000001</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="str">
+        <x:v>FORMULA: SUM(D2:D23)</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -774,7 +776,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -791,7 +793,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E3" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -808,7 +810,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E4" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -825,7 +827,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -842,7 +844,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -859,7 +861,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -876,7 +878,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E8" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -893,7 +895,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E9" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -910,7 +912,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E10" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -927,7 +929,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E11" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -944,7 +946,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E12" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -961,7 +963,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E13" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -978,7 +980,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -995,7 +997,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E15" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1012,7 +1014,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1029,7 +1031,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E17" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1046,7 +1048,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E18" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1063,7 +1065,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E19" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1080,7 +1082,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E20" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1097,7 +1099,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E21" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1114,7 +1116,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E22" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1131,7 +1133,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E23" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1148,7 +1150,7 @@
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="E24" s="7" t="str">
-        <x:v>Trang giá mở ngày 2026-10-16; cập nhật lại screenshot trước khi nộp nếu AWS thay đổi SKU.</x:v>
+        <x:v>PENDING_VERIFICATION: link chính thức để đối chiếu; chưa nhúng ảnh chụp raster, cần chụp SKU/region/đơn giá trước khi nộp.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>